<commit_message>
p y q, problema con la escala
</commit_message>
<xml_diff>
--- a/solar_nips_test.xlsx
+++ b/solar_nips_test.xlsx
@@ -646,13 +646,13 @@
         <v>55</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -666,13 +666,13 @@
         <v>55</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -689,10 +689,10 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>0.9473684210526316</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -709,10 +709,10 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="F14" t="n">
-        <v>0.888888888888889</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="15">
@@ -729,10 +729,10 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7499999999999999</v>
+        <v>0.8235294117647058</v>
       </c>
     </row>
     <row r="16">
@@ -766,13 +766,13 @@
         <v>60</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="18">
@@ -786,13 +786,13 @@
         <v>60</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="19">
@@ -806,13 +806,13 @@
         <v>60</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="20">
@@ -826,13 +826,13 @@
         <v>60</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="21">
@@ -846,13 +846,13 @@
         <v>60</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="22">
@@ -866,13 +866,13 @@
         <v>60</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0.9473684210526316</v>
       </c>
     </row>
     <row r="23">
@@ -909,10 +909,10 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>0.8888888888888888</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>0.9411764705882353</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -929,10 +929,10 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>0.8888888888888888</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>0.9411764705882353</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -949,10 +949,10 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>0.8888888888888888</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>0.9411764705882353</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -969,10 +969,10 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -989,10 +989,10 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6153846153846153</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="29">
@@ -1009,10 +1009,10 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="F29" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="30">
@@ -1026,13 +1026,13 @@
         <v>65</v>
       </c>
       <c r="D30" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.7</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>0.8750000000000001</v>
+        <v>0.8235294117647058</v>
       </c>
     </row>
     <row r="31">
@@ -1046,13 +1046,13 @@
         <v>65</v>
       </c>
       <c r="D31" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.7</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>0.8750000000000001</v>
+        <v>0.8235294117647058</v>
       </c>
     </row>
     <row r="32">
@@ -1066,13 +1066,13 @@
         <v>65</v>
       </c>
       <c r="D32" t="n">
-        <v>0.75</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E32" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="33">
@@ -1086,13 +1086,13 @@
         <v>65</v>
       </c>
       <c r="D33" t="n">
-        <v>0.75</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E33" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="34">
@@ -1106,13 +1106,13 @@
         <v>65</v>
       </c>
       <c r="D34" t="n">
-        <v>0.75</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E34" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -1126,13 +1126,13 @@
         <v>65</v>
       </c>
       <c r="D35" t="n">
-        <v>0.75</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E35" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="36">
@@ -1146,13 +1146,13 @@
         <v>65</v>
       </c>
       <c r="D36" t="n">
-        <v>0.75</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E36" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="37">
@@ -1166,13 +1166,13 @@
         <v>65</v>
       </c>
       <c r="D37" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E37" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1186,13 +1186,13 @@
         <v>65</v>
       </c>
       <c r="D38" t="n">
-        <v>0.8</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E38" t="n">
-        <v>0.5714285714285714</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8750000000000001</v>
       </c>
     </row>
     <row r="39">
@@ -1206,13 +1206,13 @@
         <v>65</v>
       </c>
       <c r="D39" t="n">
-        <v>0.8</v>
+        <v>0.875</v>
       </c>
       <c r="E39" t="n">
-        <v>0.5714285714285714</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.9333333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -1226,13 +1226,13 @@
         <v>65</v>
       </c>
       <c r="D40" t="n">
-        <v>0.8</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E40" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="F40" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="41">
@@ -1249,10 +1249,10 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F41" t="n">
-        <v>0.6</v>
+        <v>0.7272727272727273</v>
       </c>
     </row>
     <row r="42">
@@ -1266,13 +1266,13 @@
         <v>65</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="43">
@@ -1306,13 +1306,13 @@
         <v>70</v>
       </c>
       <c r="D44" t="n">
-        <v>0.625</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E44" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="45">
@@ -1326,13 +1326,13 @@
         <v>70</v>
       </c>
       <c r="D45" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E45" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7692307692307692</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="46">
@@ -1346,13 +1346,13 @@
         <v>70</v>
       </c>
       <c r="D46" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.75</v>
       </c>
       <c r="E46" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="47">
@@ -1366,13 +1366,13 @@
         <v>70</v>
       </c>
       <c r="D47" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="E47" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="48">
@@ -1386,13 +1386,13 @@
         <v>70</v>
       </c>
       <c r="D48" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="E48" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="49">
@@ -1406,13 +1406,13 @@
         <v>70</v>
       </c>
       <c r="D49" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="E49" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="50">
@@ -1426,13 +1426,13 @@
         <v>70</v>
       </c>
       <c r="D50" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="E50" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="51">
@@ -1446,13 +1446,13 @@
         <v>70</v>
       </c>
       <c r="D51" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E51" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F51" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.7692307692307692</v>
       </c>
     </row>
     <row r="52">
@@ -1466,13 +1466,13 @@
         <v>70</v>
       </c>
       <c r="D52" t="n">
-        <v>0.5</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E52" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F52" t="n">
-        <v>0.25</v>
+        <v>0.7692307692307692</v>
       </c>
     </row>
     <row r="53">
@@ -1486,13 +1486,13 @@
         <v>70</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="54">
@@ -1506,13 +1506,13 @@
         <v>70</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>0</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="55">
@@ -1586,13 +1586,13 @@
         <v>75</v>
       </c>
       <c r="D58" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E58" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>0.4444444444444445</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="59">
@@ -1606,13 +1606,13 @@
         <v>75</v>
       </c>
       <c r="D59" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E59" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>0.4444444444444445</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="60">
@@ -1626,13 +1626,13 @@
         <v>75</v>
       </c>
       <c r="D60" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E60" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>0.25</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="61">
@@ -1646,13 +1646,13 @@
         <v>75</v>
       </c>
       <c r="D61" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="E61" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>0.2857142857142858</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="62">
@@ -1666,13 +1666,13 @@
         <v>75</v>
       </c>
       <c r="D62" t="n">
-        <v>0.5</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="E62" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.7272727272727273</v>
       </c>
     </row>
     <row r="63">
@@ -1686,13 +1686,13 @@
         <v>75</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="E63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>0.7272727272727273</v>
       </c>
     </row>
     <row r="64">
@@ -1706,13 +1706,13 @@
         <v>75</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E64" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="65">
@@ -1726,13 +1726,13 @@
         <v>75</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E65" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="66">
@@ -1869,10 +1869,10 @@
         <v>0.5</v>
       </c>
       <c r="E72" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="73">
@@ -1886,13 +1886,13 @@
         <v>80</v>
       </c>
       <c r="D73" t="n">
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="E73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>0</v>
+        <v>0.7272727272727273</v>
       </c>
     </row>
     <row r="74">
@@ -1906,13 +1906,13 @@
         <v>80</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="75">
@@ -1926,13 +1926,13 @@
         <v>80</v>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="76">
@@ -1946,13 +1946,13 @@
         <v>80</v>
       </c>
       <c r="D76" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E76" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F76" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="77">
@@ -2146,13 +2146,13 @@
         <v>85</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="E86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="87">
@@ -2166,13 +2166,13 @@
         <v>85</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F87" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="88">

</xml_diff>